<commit_message>
launch-content: posts organised by day and post in one ZIP, bundle graphics, safe-zone fixes
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/launch-content/plan/11_a_Day_Schedule.xlsx
+++ b/launch-content/plan/11_a_Day_Schedule.xlsx
@@ -519,7 +519,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>The file names match files in the 01_ALL_POSTS_IN_ONE_FOLDER folder, and each has a matching .txt caption.</t>
+          <t>Each row names the post folder inside 01_POSTS_BY_DAY/Day_XX. Open it: the image or video and Caption.txt are together.</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>File name(s)</t>
+          <t>Post folder (inside the Day folder)</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>O01_Carousel1_Slide1.png, O01_Carousel1_Slide2.png, O01_Carousel1_Slide3.png, O01_Carousel1_Slide4.png, O01_Carousel1_Slide5.png, O01_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>O01_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>O01_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>O01_Video1_Price-question.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>O01_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr"/>
@@ -963,7 +963,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>O01_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>O01_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>O01_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr"/>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>O01_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr"/>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>O01_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr"/>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>ALL_Nine_Offers_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_All-nine-launch-banner</t>
         </is>
       </c>
       <c r="J16" s="9" t="inlineStr"/>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>O02_Carousel1_Slide1.png, O02_Carousel1_Slide2.png, O02_Carousel1_Slide3.png, O02_Carousel1_Slide4.png, O02_Carousel1_Slide5.png, O02_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr"/>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>O02_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr"/>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>O02_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>O02_Video1_Ten-second-test.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr"/>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>O02_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr"/>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>O02_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>O02_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>O02_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr"/>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>O02_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr"/>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>O02_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr"/>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>O02_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr"/>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>O03_Carousel1_Slide1.png, O03_Carousel1_Slide2.png, O03_Carousel1_Slide3.png, O03_Carousel1_Slide4.png, O03_Carousel1_Slide5.png, O03_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr"/>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>O03_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr"/>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>O03_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr"/>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>O03_Video1_Four-pillars.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>O03_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr"/>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>O03_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>O03_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J34" s="9" t="inlineStr"/>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>O03_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J35" s="9" t="inlineStr"/>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>O03_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J36" s="9" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>O03_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J37" s="9" t="inlineStr"/>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>O03_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J38" s="9" t="inlineStr"/>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>O04_Carousel1_Slide1.png, O04_Carousel1_Slide2.png, O04_Carousel1_Slide3.png, O04_Carousel1_Slide4.png, O04_Carousel1_Slide5.png, O04_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J39" s="9" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>O04_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr"/>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>O04_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr"/>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>O04_Video1_One-offer-one-page.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J42" s="9" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>O04_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J43" s="9" t="inlineStr"/>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>O04_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J44" s="9" t="inlineStr"/>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>O04_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J45" s="9" t="inlineStr"/>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>O04_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J46" s="9" t="inlineStr"/>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>O04_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J47" s="9" t="inlineStr"/>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>O04_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J48" s="9" t="inlineStr"/>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>O04_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J49" s="9" t="inlineStr"/>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>O05_Carousel1_Slide1.png, O05_Carousel1_Slide2.png, O05_Carousel1_Slide3.png, O05_Carousel1_Slide4.png, O05_Carousel1_Slide5.png, O05_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J50" s="9" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>O05_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J51" s="9" t="inlineStr"/>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>O05_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J52" s="9" t="inlineStr"/>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>O05_Video1_Search-yourself.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J53" s="9" t="inlineStr"/>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>O05_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr"/>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>O05_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J55" s="9" t="inlineStr"/>
@@ -3168,7 +3168,7 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>O05_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J56" s="9" t="inlineStr"/>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>O05_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J57" s="9" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>O05_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J58" s="9" t="inlineStr"/>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>O05_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J59" s="9" t="inlineStr"/>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>O05_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J60" s="9" t="inlineStr"/>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>O06_Carousel1_Slide1.png, O06_Carousel1_Slide2.png, O06_Carousel1_Slide3.png, O06_Carousel1_Slide4.png, O06_Carousel1_Slide5.png, O06_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J61" s="9" t="inlineStr"/>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>O06_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J62" s="9" t="inlineStr"/>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>O06_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J63" s="9" t="inlineStr"/>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>O06_Video1_One-sentence.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J64" s="9" t="inlineStr"/>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>O06_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J65" s="9" t="inlineStr"/>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>O06_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J66" s="9" t="inlineStr"/>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>O06_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J67" s="9" t="inlineStr"/>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
-          <t>O06_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J68" s="9" t="inlineStr"/>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>O06_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J69" s="9" t="inlineStr"/>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>O06_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr"/>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>O06_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr"/>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="I72" s="7" t="inlineStr">
         <is>
-          <t>O07_Carousel1_Slide1.png, O07_Carousel1_Slide2.png, O07_Carousel1_Slide3.png, O07_Carousel1_Slide4.png, O07_Carousel1_Slide5.png, O07_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr"/>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>O07_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr"/>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>O07_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr"/>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>O07_Video1_Five-part-prompt.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J75" s="9" t="inlineStr"/>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
-          <t>O07_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J76" s="9" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>O07_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J77" s="9" t="inlineStr"/>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>O07_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J78" s="9" t="inlineStr"/>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>O07_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J79" s="9" t="inlineStr"/>
@@ -4344,7 +4344,7 @@
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>O07_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J80" s="9" t="inlineStr"/>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>O07_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr"/>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>O07_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J82" s="9" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>O08_Carousel1_Slide1.png, O08_Carousel1_Slide2.png, O08_Carousel1_Slide3.png, O08_Carousel1_Slide4.png, O08_Carousel1_Slide5.png, O08_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J83" s="9" t="inlineStr"/>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>O08_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J84" s="9" t="inlineStr"/>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>O08_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J85" s="9" t="inlineStr"/>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
-          <t>O08_Video1_One-page-rule.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J86" s="9" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
-          <t>O08_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J87" s="9" t="inlineStr"/>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="I88" s="7" t="inlineStr">
         <is>
-          <t>O08_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J88" s="9" t="inlineStr"/>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>O08_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J89" s="9" t="inlineStr"/>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
-          <t>O08_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J90" s="9" t="inlineStr"/>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>O08_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J91" s="9" t="inlineStr"/>
@@ -4932,7 +4932,7 @@
       </c>
       <c r="I92" s="7" t="inlineStr">
         <is>
-          <t>O08_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J92" s="9" t="inlineStr"/>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
-          <t>O08_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J93" s="9" t="inlineStr"/>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="I94" s="7" t="inlineStr">
         <is>
-          <t>O09_Carousel1_Slide1.png, O09_Carousel1_Slide2.png, O09_Carousel1_Slide3.png, O09_Carousel1_Slide4.png, O09_Carousel1_Slide5.png, O09_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J94" s="9" t="inlineStr"/>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
-          <t>O09_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J95" s="9" t="inlineStr"/>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="I96" s="7" t="inlineStr">
         <is>
-          <t>O09_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J96" s="9" t="inlineStr"/>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
-          <t>O09_Video1_Own-your-domain.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J97" s="9" t="inlineStr"/>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="I98" s="7" t="inlineStr">
         <is>
-          <t>O09_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J98" s="9" t="inlineStr"/>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>O09_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J99" s="9" t="inlineStr"/>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="I100" s="7" t="inlineStr">
         <is>
-          <t>O09_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J100" s="9" t="inlineStr"/>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="I101" s="7" t="inlineStr">
         <is>
-          <t>O09_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J101" s="9" t="inlineStr"/>
@@ -5422,7 +5422,7 @@
       </c>
       <c r="I102" s="7" t="inlineStr">
         <is>
-          <t>O09_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J102" s="9" t="inlineStr"/>
@@ -5471,7 +5471,7 @@
       </c>
       <c r="I103" s="7" t="inlineStr">
         <is>
-          <t>O09_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J103" s="9" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="I104" s="7" t="inlineStr">
         <is>
-          <t>O09_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J104" s="9" t="inlineStr"/>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="I105" s="7" t="inlineStr">
         <is>
-          <t>O01_Carousel2_Slide1.png, O01_Carousel2_Slide2.png, O01_Carousel2_Slide3.png, O01_Carousel2_Slide4.png, O01_Carousel2_Slide5.png, O01_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J105" s="9" t="inlineStr"/>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="I106" s="7" t="inlineStr">
         <is>
-          <t>O01_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J106" s="9" t="inlineStr"/>
@@ -5667,7 +5667,7 @@
       </c>
       <c r="I107" s="7" t="inlineStr">
         <is>
-          <t>O01_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J107" s="9" t="inlineStr"/>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="I108" s="7" t="inlineStr">
         <is>
-          <t>O01_Video2_Follow-up-rhythm.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J108" s="9" t="inlineStr"/>
@@ -5765,7 +5765,7 @@
       </c>
       <c r="I109" s="7" t="inlineStr">
         <is>
-          <t>O01_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J109" s="9" t="inlineStr"/>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I110" s="7" t="inlineStr">
         <is>
-          <t>O01_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J110" s="9" t="inlineStr"/>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="I111" s="7" t="inlineStr">
         <is>
-          <t>O01_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J111" s="9" t="inlineStr"/>
@@ -5912,7 +5912,7 @@
       </c>
       <c r="I112" s="7" t="inlineStr">
         <is>
-          <t>O01_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J112" s="9" t="inlineStr"/>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="I113" s="7" t="inlineStr">
         <is>
-          <t>O01_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J113" s="9" t="inlineStr"/>
@@ -6010,7 +6010,7 @@
       </c>
       <c r="I114" s="7" t="inlineStr">
         <is>
-          <t>O01_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J114" s="9" t="inlineStr"/>
@@ -6059,7 +6059,7 @@
       </c>
       <c r="I115" s="7" t="inlineStr">
         <is>
-          <t>O01_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J115" s="9" t="inlineStr"/>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="I116" s="7" t="inlineStr">
         <is>
-          <t>O02_Carousel2_Slide1.png, O02_Carousel2_Slide2.png, O02_Carousel2_Slide3.png, O02_Carousel2_Slide4.png, O02_Carousel2_Slide5.png, O02_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J116" s="9" t="inlineStr"/>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="I117" s="7" t="inlineStr">
         <is>
-          <t>O02_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J117" s="9" t="inlineStr"/>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="I118" s="7" t="inlineStr">
         <is>
-          <t>O02_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J118" s="9" t="inlineStr"/>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I119" s="7" t="inlineStr">
         <is>
-          <t>O02_Video2_Headline-fix.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J119" s="9" t="inlineStr"/>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="I120" s="7" t="inlineStr">
         <is>
-          <t>O02_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J120" s="9" t="inlineStr"/>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="I121" s="7" t="inlineStr">
         <is>
-          <t>O02_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J121" s="9" t="inlineStr"/>
@@ -6402,7 +6402,7 @@
       </c>
       <c r="I122" s="7" t="inlineStr">
         <is>
-          <t>O02_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J122" s="9" t="inlineStr"/>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="I123" s="7" t="inlineStr">
         <is>
-          <t>O02_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J123" s="9" t="inlineStr"/>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="I124" s="7" t="inlineStr">
         <is>
-          <t>O02_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J124" s="9" t="inlineStr"/>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="I125" s="7" t="inlineStr">
         <is>
-          <t>O02_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J125" s="9" t="inlineStr"/>
@@ -6598,7 +6598,7 @@
       </c>
       <c r="I126" s="7" t="inlineStr">
         <is>
-          <t>O02_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J126" s="9" t="inlineStr"/>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="I127" s="7" t="inlineStr">
         <is>
-          <t>O03_Carousel2_Slide1.png, O03_Carousel2_Slide2.png, O03_Carousel2_Slide3.png, O03_Carousel2_Slide4.png, O03_Carousel2_Slide5.png, O03_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J127" s="9" t="inlineStr"/>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="I128" s="7" t="inlineStr">
         <is>
-          <t>O03_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J128" s="9" t="inlineStr"/>
@@ -6745,7 +6745,7 @@
       </c>
       <c r="I129" s="7" t="inlineStr">
         <is>
-          <t>O03_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J129" s="9" t="inlineStr"/>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="I130" s="7" t="inlineStr">
         <is>
-          <t>O03_Video2_Batching.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J130" s="9" t="inlineStr"/>
@@ -6843,7 +6843,7 @@
       </c>
       <c r="I131" s="7" t="inlineStr">
         <is>
-          <t>O03_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J131" s="9" t="inlineStr"/>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="I132" s="7" t="inlineStr">
         <is>
-          <t>O03_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J132" s="9" t="inlineStr"/>
@@ -6941,7 +6941,7 @@
       </c>
       <c r="I133" s="7" t="inlineStr">
         <is>
-          <t>O03_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J133" s="9" t="inlineStr"/>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="I134" s="7" t="inlineStr">
         <is>
-          <t>O03_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J134" s="9" t="inlineStr"/>
@@ -7039,7 +7039,7 @@
       </c>
       <c r="I135" s="7" t="inlineStr">
         <is>
-          <t>O03_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J135" s="9" t="inlineStr"/>
@@ -7088,7 +7088,7 @@
       </c>
       <c r="I136" s="7" t="inlineStr">
         <is>
-          <t>O03_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J136" s="9" t="inlineStr"/>
@@ -7137,7 +7137,7 @@
       </c>
       <c r="I137" s="7" t="inlineStr">
         <is>
-          <t>O03_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J137" s="9" t="inlineStr"/>
@@ -7186,7 +7186,7 @@
       </c>
       <c r="I138" s="7" t="inlineStr">
         <is>
-          <t>O04_Carousel2_Slide1.png, O04_Carousel2_Slide2.png, O04_Carousel2_Slide3.png, O04_Carousel2_Slide4.png, O04_Carousel2_Slide5.png, O04_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J138" s="9" t="inlineStr"/>
@@ -7235,7 +7235,7 @@
       </c>
       <c r="I139" s="7" t="inlineStr">
         <is>
-          <t>O04_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J139" s="9" t="inlineStr"/>
@@ -7284,7 +7284,7 @@
       </c>
       <c r="I140" s="7" t="inlineStr">
         <is>
-          <t>O04_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J140" s="9" t="inlineStr"/>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="I141" s="7" t="inlineStr">
         <is>
-          <t>O04_Video2_Phone-check.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J141" s="9" t="inlineStr"/>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="I142" s="7" t="inlineStr">
         <is>
-          <t>O04_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J142" s="9" t="inlineStr"/>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="I143" s="7" t="inlineStr">
         <is>
-          <t>O04_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J143" s="9" t="inlineStr"/>
@@ -7480,7 +7480,7 @@
       </c>
       <c r="I144" s="7" t="inlineStr">
         <is>
-          <t>O04_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J144" s="9" t="inlineStr"/>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="I145" s="7" t="inlineStr">
         <is>
-          <t>O04_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J145" s="9" t="inlineStr"/>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="I146" s="7" t="inlineStr">
         <is>
-          <t>O04_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J146" s="9" t="inlineStr"/>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="I147" s="7" t="inlineStr">
         <is>
-          <t>O04_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J147" s="9" t="inlineStr"/>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="I148" s="7" t="inlineStr">
         <is>
-          <t>O04_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J148" s="9" t="inlineStr"/>
@@ -7725,7 +7725,7 @@
       </c>
       <c r="I149" s="7" t="inlineStr">
         <is>
-          <t>O05_Carousel2_Slide1.png, O05_Carousel2_Slide2.png, O05_Carousel2_Slide3.png, O05_Carousel2_Slide4.png, O05_Carousel2_Slide5.png, O05_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J149" s="9" t="inlineStr"/>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="I150" s="7" t="inlineStr">
         <is>
-          <t>O05_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J150" s="9" t="inlineStr"/>
@@ -7823,7 +7823,7 @@
       </c>
       <c r="I151" s="7" t="inlineStr">
         <is>
-          <t>O05_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J151" s="9" t="inlineStr"/>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="I152" s="7" t="inlineStr">
         <is>
-          <t>O05_Video2_Reviews.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J152" s="9" t="inlineStr"/>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="I153" s="7" t="inlineStr">
         <is>
-          <t>O05_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J153" s="9" t="inlineStr"/>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="I154" s="7" t="inlineStr">
         <is>
-          <t>O05_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J154" s="9" t="inlineStr"/>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="I155" s="7" t="inlineStr">
         <is>
-          <t>O05_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J155" s="9" t="inlineStr"/>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="I156" s="7" t="inlineStr">
         <is>
-          <t>O05_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J156" s="9" t="inlineStr"/>
@@ -8117,7 +8117,7 @@
       </c>
       <c r="I157" s="7" t="inlineStr">
         <is>
-          <t>O05_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J157" s="9" t="inlineStr"/>
@@ -8166,7 +8166,7 @@
       </c>
       <c r="I158" s="7" t="inlineStr">
         <is>
-          <t>O05_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J158" s="9" t="inlineStr"/>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="I159" s="7" t="inlineStr">
         <is>
-          <t>O05_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J159" s="9" t="inlineStr"/>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="I160" s="7" t="inlineStr">
         <is>
-          <t>O06_Carousel2_Slide1.png, O06_Carousel2_Slide2.png, O06_Carousel2_Slide3.png, O06_Carousel2_Slide4.png, O06_Carousel2_Slide5.png, O06_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J160" s="9" t="inlineStr"/>
@@ -8313,7 +8313,7 @@
       </c>
       <c r="I161" s="7" t="inlineStr">
         <is>
-          <t>O06_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J161" s="9" t="inlineStr"/>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="I162" s="7" t="inlineStr">
         <is>
-          <t>O06_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J162" s="9" t="inlineStr"/>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="I163" s="7" t="inlineStr">
         <is>
-          <t>O06_Video2_Ask-five-customers.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J163" s="9" t="inlineStr"/>
@@ -8460,7 +8460,7 @@
       </c>
       <c r="I164" s="7" t="inlineStr">
         <is>
-          <t>O06_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J164" s="9" t="inlineStr"/>
@@ -8509,7 +8509,7 @@
       </c>
       <c r="I165" s="7" t="inlineStr">
         <is>
-          <t>O06_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J165" s="9" t="inlineStr"/>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="I166" s="7" t="inlineStr">
         <is>
-          <t>O06_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J166" s="9" t="inlineStr"/>
@@ -8607,7 +8607,7 @@
       </c>
       <c r="I167" s="7" t="inlineStr">
         <is>
-          <t>O06_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J167" s="9" t="inlineStr"/>
@@ -8656,7 +8656,7 @@
       </c>
       <c r="I168" s="7" t="inlineStr">
         <is>
-          <t>O06_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J168" s="9" t="inlineStr"/>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="I169" s="7" t="inlineStr">
         <is>
-          <t>O06_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J169" s="9" t="inlineStr"/>
@@ -8754,7 +8754,7 @@
       </c>
       <c r="I170" s="7" t="inlineStr">
         <is>
-          <t>O06_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J170" s="9" t="inlineStr"/>
@@ -8803,7 +8803,7 @@
       </c>
       <c r="I171" s="7" t="inlineStr">
         <is>
-          <t>O07_Carousel2_Slide1.png, O07_Carousel2_Slide2.png, O07_Carousel2_Slide3.png, O07_Carousel2_Slide4.png, O07_Carousel2_Slide5.png, O07_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J171" s="9" t="inlineStr"/>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="I172" s="7" t="inlineStr">
         <is>
-          <t>O07_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J172" s="9" t="inlineStr"/>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="I173" s="7" t="inlineStr">
         <is>
-          <t>O07_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J173" s="9" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="I174" s="7" t="inlineStr">
         <is>
-          <t>O07_Video2_Never-paste.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J174" s="9" t="inlineStr"/>
@@ -8999,7 +8999,7 @@
       </c>
       <c r="I175" s="7" t="inlineStr">
         <is>
-          <t>O07_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J175" s="9" t="inlineStr"/>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="I176" s="7" t="inlineStr">
         <is>
-          <t>O07_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J176" s="9" t="inlineStr"/>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="I177" s="7" t="inlineStr">
         <is>
-          <t>O07_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J177" s="9" t="inlineStr"/>
@@ -9146,7 +9146,7 @@
       </c>
       <c r="I178" s="7" t="inlineStr">
         <is>
-          <t>O07_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J178" s="9" t="inlineStr"/>
@@ -9195,7 +9195,7 @@
       </c>
       <c r="I179" s="7" t="inlineStr">
         <is>
-          <t>O07_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J179" s="9" t="inlineStr"/>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="I180" s="7" t="inlineStr">
         <is>
-          <t>O07_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J180" s="9" t="inlineStr"/>
@@ -9293,7 +9293,7 @@
       </c>
       <c r="I181" s="7" t="inlineStr">
         <is>
-          <t>O07_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J181" s="9" t="inlineStr"/>
@@ -9342,7 +9342,7 @@
       </c>
       <c r="I182" s="7" t="inlineStr">
         <is>
-          <t>O08_Carousel2_Slide1.png, O08_Carousel2_Slide2.png, O08_Carousel2_Slide3.png, O08_Carousel2_Slide4.png, O08_Carousel2_Slide5.png, O08_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J182" s="9" t="inlineStr"/>
@@ -9391,7 +9391,7 @@
       </c>
       <c r="I183" s="7" t="inlineStr">
         <is>
-          <t>O08_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J183" s="9" t="inlineStr"/>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="I184" s="7" t="inlineStr">
         <is>
-          <t>O08_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J184" s="9" t="inlineStr"/>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="I185" s="7" t="inlineStr">
         <is>
-          <t>O08_Video2_Price-options.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J185" s="9" t="inlineStr"/>
@@ -9538,7 +9538,7 @@
       </c>
       <c r="I186" s="7" t="inlineStr">
         <is>
-          <t>O08_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J186" s="9" t="inlineStr"/>
@@ -9587,7 +9587,7 @@
       </c>
       <c r="I187" s="7" t="inlineStr">
         <is>
-          <t>O08_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J187" s="9" t="inlineStr"/>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="I188" s="7" t="inlineStr">
         <is>
-          <t>O08_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J188" s="9" t="inlineStr"/>
@@ -9685,7 +9685,7 @@
       </c>
       <c r="I189" s="7" t="inlineStr">
         <is>
-          <t>O08_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J189" s="9" t="inlineStr"/>
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I190" s="7" t="inlineStr">
         <is>
-          <t>O08_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J190" s="9" t="inlineStr"/>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="I191" s="7" t="inlineStr">
         <is>
-          <t>O08_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J191" s="9" t="inlineStr"/>
@@ -9832,7 +9832,7 @@
       </c>
       <c r="I192" s="7" t="inlineStr">
         <is>
-          <t>O08_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J192" s="9" t="inlineStr"/>
@@ -9881,7 +9881,7 @@
       </c>
       <c r="I193" s="7" t="inlineStr">
         <is>
-          <t>O09_Carousel2_Slide1.png, O09_Carousel2_Slide2.png, O09_Carousel2_Slide3.png, O09_Carousel2_Slide4.png, O09_Carousel2_Slide5.png, O09_Carousel2_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J193" s="9" t="inlineStr"/>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="I194" s="7" t="inlineStr">
         <is>
-          <t>O09_Post10_Whats-inside.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J194" s="9" t="inlineStr"/>
@@ -9979,7 +9979,7 @@
       </c>
       <c r="I195" s="7" t="inlineStr">
         <is>
-          <t>O09_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J195" s="9" t="inlineStr"/>
@@ -10028,7 +10028,7 @@
       </c>
       <c r="I196" s="7" t="inlineStr">
         <is>
-          <t>O09_Video2_Monthly-check.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J196" s="9" t="inlineStr"/>
@@ -10077,7 +10077,7 @@
       </c>
       <c r="I197" s="7" t="inlineStr">
         <is>
-          <t>O09_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J197" s="9" t="inlineStr"/>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="I198" s="7" t="inlineStr">
         <is>
-          <t>O09_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J198" s="9" t="inlineStr"/>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="I199" s="7" t="inlineStr">
         <is>
-          <t>O09_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J199" s="9" t="inlineStr"/>
@@ -10224,7 +10224,7 @@
       </c>
       <c r="I200" s="7" t="inlineStr">
         <is>
-          <t>O09_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J200" s="9" t="inlineStr"/>
@@ -10273,7 +10273,7 @@
       </c>
       <c r="I201" s="7" t="inlineStr">
         <is>
-          <t>O09_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J201" s="9" t="inlineStr"/>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="I202" s="7" t="inlineStr">
         <is>
-          <t>O09_Post04_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J202" s="9" t="inlineStr"/>
@@ -10371,7 +10371,7 @@
       </c>
       <c r="I203" s="7" t="inlineStr">
         <is>
-          <t>O09_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J203" s="9" t="inlineStr"/>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="I204" s="7" t="inlineStr">
         <is>
-          <t>O01_Carousel3_Slide1.png, O01_Carousel3_Slide2.png, O01_Carousel3_Slide3.png, O01_Carousel3_Slide4.png, O01_Carousel3_Slide5.png, O01_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J204" s="9" t="inlineStr"/>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="I205" s="7" t="inlineStr">
         <is>
-          <t>O01_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J205" s="9" t="inlineStr"/>
@@ -10518,7 +10518,7 @@
       </c>
       <c r="I206" s="7" t="inlineStr">
         <is>
-          <t>O01_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J206" s="9" t="inlineStr"/>
@@ -10567,7 +10567,7 @@
       </c>
       <c r="I207" s="7" t="inlineStr">
         <is>
-          <t>O01_Video3_Your-chat-is-your-shop.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J207" s="9" t="inlineStr"/>
@@ -10616,7 +10616,7 @@
       </c>
       <c r="I208" s="7" t="inlineStr">
         <is>
-          <t>O01_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J208" s="9" t="inlineStr"/>
@@ -10665,7 +10665,7 @@
       </c>
       <c r="I209" s="7" t="inlineStr">
         <is>
-          <t>O01_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J209" s="9" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="I210" s="7" t="inlineStr">
         <is>
-          <t>O01_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J210" s="9" t="inlineStr"/>
@@ -10763,7 +10763,7 @@
       </c>
       <c r="I211" s="7" t="inlineStr">
         <is>
-          <t>O01_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J211" s="9" t="inlineStr"/>
@@ -10812,7 +10812,7 @@
       </c>
       <c r="I212" s="7" t="inlineStr">
         <is>
-          <t>O01_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J212" s="9" t="inlineStr"/>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="I213" s="7" t="inlineStr">
         <is>
-          <t>O01_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J213" s="9" t="inlineStr"/>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="I214" s="7" t="inlineStr">
         <is>
-          <t>O01_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J214" s="9" t="inlineStr"/>
@@ -10959,7 +10959,7 @@
       </c>
       <c r="I215" s="7" t="inlineStr">
         <is>
-          <t>O02_Carousel3_Slide1.png, O02_Carousel3_Slide2.png, O02_Carousel3_Slide3.png, O02_Carousel3_Slide4.png, O02_Carousel3_Slide5.png, O02_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J215" s="9" t="inlineStr"/>
@@ -11008,7 +11008,7 @@
       </c>
       <c r="I216" s="7" t="inlineStr">
         <is>
-          <t>O02_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J216" s="9" t="inlineStr"/>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="I217" s="7" t="inlineStr">
         <is>
-          <t>O02_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J217" s="9" t="inlineStr"/>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="I218" s="7" t="inlineStr">
         <is>
-          <t>O02_Video3_One-button.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J218" s="9" t="inlineStr"/>
@@ -11155,7 +11155,7 @@
       </c>
       <c r="I219" s="7" t="inlineStr">
         <is>
-          <t>O02_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J219" s="9" t="inlineStr"/>
@@ -11204,7 +11204,7 @@
       </c>
       <c r="I220" s="7" t="inlineStr">
         <is>
-          <t>O02_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J220" s="9" t="inlineStr"/>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="I221" s="7" t="inlineStr">
         <is>
-          <t>O02_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J221" s="9" t="inlineStr"/>
@@ -11302,7 +11302,7 @@
       </c>
       <c r="I222" s="7" t="inlineStr">
         <is>
-          <t>O02_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J222" s="9" t="inlineStr"/>
@@ -11351,7 +11351,7 @@
       </c>
       <c r="I223" s="7" t="inlineStr">
         <is>
-          <t>O02_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J223" s="9" t="inlineStr"/>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="I224" s="7" t="inlineStr">
         <is>
-          <t>O02_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J224" s="9" t="inlineStr"/>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="I225" s="7" t="inlineStr">
         <is>
-          <t>O02_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J225" s="9" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="I226" s="7" t="inlineStr">
         <is>
-          <t>O03_Carousel3_Slide1.png, O03_Carousel3_Slide2.png, O03_Carousel3_Slide3.png, O03_Carousel3_Slide4.png, O03_Carousel3_Slide5.png, O03_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J226" s="9" t="inlineStr"/>
@@ -11547,7 +11547,7 @@
       </c>
       <c r="I227" s="7" t="inlineStr">
         <is>
-          <t>O03_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J227" s="9" t="inlineStr"/>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="I228" s="7" t="inlineStr">
         <is>
-          <t>O03_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J228" s="9" t="inlineStr"/>
@@ -11645,7 +11645,7 @@
       </c>
       <c r="I229" s="7" t="inlineStr">
         <is>
-          <t>O03_Video3_Hooks.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J229" s="9" t="inlineStr"/>
@@ -11694,7 +11694,7 @@
       </c>
       <c r="I230" s="7" t="inlineStr">
         <is>
-          <t>O03_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J230" s="9" t="inlineStr"/>
@@ -11743,7 +11743,7 @@
       </c>
       <c r="I231" s="7" t="inlineStr">
         <is>
-          <t>O03_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J231" s="9" t="inlineStr"/>
@@ -11792,7 +11792,7 @@
       </c>
       <c r="I232" s="7" t="inlineStr">
         <is>
-          <t>O03_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J232" s="9" t="inlineStr"/>
@@ -11841,7 +11841,7 @@
       </c>
       <c r="I233" s="7" t="inlineStr">
         <is>
-          <t>O03_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J233" s="9" t="inlineStr"/>
@@ -11890,7 +11890,7 @@
       </c>
       <c r="I234" s="7" t="inlineStr">
         <is>
-          <t>O03_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J234" s="9" t="inlineStr"/>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="I235" s="7" t="inlineStr">
         <is>
-          <t>O03_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J235" s="9" t="inlineStr"/>
@@ -11988,7 +11988,7 @@
       </c>
       <c r="I236" s="7" t="inlineStr">
         <is>
-          <t>O03_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J236" s="9" t="inlineStr"/>
@@ -12037,7 +12037,7 @@
       </c>
       <c r="I237" s="7" t="inlineStr">
         <is>
-          <t>O04_Carousel3_Slide1.png, O04_Carousel3_Slide2.png, O04_Carousel3_Slide3.png, O04_Carousel3_Slide4.png, O04_Carousel3_Slide5.png, O04_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J237" s="9" t="inlineStr"/>
@@ -12086,7 +12086,7 @@
       </c>
       <c r="I238" s="7" t="inlineStr">
         <is>
-          <t>O04_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J238" s="9" t="inlineStr"/>
@@ -12135,7 +12135,7 @@
       </c>
       <c r="I239" s="7" t="inlineStr">
         <is>
-          <t>O04_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J239" s="9" t="inlineStr"/>
@@ -12184,7 +12184,7 @@
       </c>
       <c r="I240" s="7" t="inlineStr">
         <is>
-          <t>O04_Video3_Honest-scope.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J240" s="9" t="inlineStr"/>
@@ -12233,7 +12233,7 @@
       </c>
       <c r="I241" s="7" t="inlineStr">
         <is>
-          <t>O04_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J241" s="9" t="inlineStr"/>
@@ -12282,7 +12282,7 @@
       </c>
       <c r="I242" s="7" t="inlineStr">
         <is>
-          <t>O04_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J242" s="9" t="inlineStr"/>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="I243" s="7" t="inlineStr">
         <is>
-          <t>O04_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J243" s="9" t="inlineStr"/>
@@ -12380,7 +12380,7 @@
       </c>
       <c r="I244" s="7" t="inlineStr">
         <is>
-          <t>O04_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J244" s="9" t="inlineStr"/>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="I245" s="7" t="inlineStr">
         <is>
-          <t>O04_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J245" s="9" t="inlineStr"/>
@@ -12478,7 +12478,7 @@
       </c>
       <c r="I246" s="7" t="inlineStr">
         <is>
-          <t>O04_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J246" s="9" t="inlineStr"/>
@@ -12527,7 +12527,7 @@
       </c>
       <c r="I247" s="7" t="inlineStr">
         <is>
-          <t>O04_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J247" s="9" t="inlineStr"/>
@@ -12576,7 +12576,7 @@
       </c>
       <c r="I248" s="7" t="inlineStr">
         <is>
-          <t>O05_Carousel3_Slide1.png, O05_Carousel3_Slide2.png, O05_Carousel3_Slide3.png, O05_Carousel3_Slide4.png, O05_Carousel3_Slide5.png, O05_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J248" s="9" t="inlineStr"/>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="I249" s="7" t="inlineStr">
         <is>
-          <t>O05_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J249" s="9" t="inlineStr"/>
@@ -12674,7 +12674,7 @@
       </c>
       <c r="I250" s="7" t="inlineStr">
         <is>
-          <t>O05_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J250" s="9" t="inlineStr"/>
@@ -12723,7 +12723,7 @@
       </c>
       <c r="I251" s="7" t="inlineStr">
         <is>
-          <t>O05_Video3_Complete-profile.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J251" s="9" t="inlineStr"/>
@@ -12772,7 +12772,7 @@
       </c>
       <c r="I252" s="7" t="inlineStr">
         <is>
-          <t>O05_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J252" s="9" t="inlineStr"/>
@@ -12821,7 +12821,7 @@
       </c>
       <c r="I253" s="7" t="inlineStr">
         <is>
-          <t>O05_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J253" s="9" t="inlineStr"/>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="I254" s="7" t="inlineStr">
         <is>
-          <t>O05_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J254" s="9" t="inlineStr"/>
@@ -12919,7 +12919,7 @@
       </c>
       <c r="I255" s="7" t="inlineStr">
         <is>
-          <t>O05_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J255" s="9" t="inlineStr"/>
@@ -12968,7 +12968,7 @@
       </c>
       <c r="I256" s="7" t="inlineStr">
         <is>
-          <t>O05_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J256" s="9" t="inlineStr"/>
@@ -13017,7 +13017,7 @@
       </c>
       <c r="I257" s="7" t="inlineStr">
         <is>
-          <t>O05_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J257" s="9" t="inlineStr"/>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="I258" s="7" t="inlineStr">
         <is>
-          <t>O05_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J258" s="9" t="inlineStr"/>
@@ -13115,7 +13115,7 @@
       </c>
       <c r="I259" s="7" t="inlineStr">
         <is>
-          <t>O06_Carousel3_Slide1.png, O06_Carousel3_Slide2.png, O06_Carousel3_Slide3.png, O06_Carousel3_Slide4.png, O06_Carousel3_Slide5.png, O06_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J259" s="9" t="inlineStr"/>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="I260" s="7" t="inlineStr">
         <is>
-          <t>O06_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J260" s="9" t="inlineStr"/>
@@ -13213,7 +13213,7 @@
       </c>
       <c r="I261" s="7" t="inlineStr">
         <is>
-          <t>O06_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J261" s="9" t="inlineStr"/>
@@ -13262,7 +13262,7 @@
       </c>
       <c r="I262" s="7" t="inlineStr">
         <is>
-          <t>O06_Video3_Not-louder-clearer.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J262" s="9" t="inlineStr"/>
@@ -13311,7 +13311,7 @@
       </c>
       <c r="I263" s="7" t="inlineStr">
         <is>
-          <t>O06_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J263" s="9" t="inlineStr"/>
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I264" s="7" t="inlineStr">
         <is>
-          <t>O06_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J264" s="9" t="inlineStr"/>
@@ -13409,7 +13409,7 @@
       </c>
       <c r="I265" s="7" t="inlineStr">
         <is>
-          <t>O06_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J265" s="9" t="inlineStr"/>
@@ -13458,7 +13458,7 @@
       </c>
       <c r="I266" s="7" t="inlineStr">
         <is>
-          <t>O06_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J266" s="9" t="inlineStr"/>
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I267" s="7" t="inlineStr">
         <is>
-          <t>O06_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J267" s="9" t="inlineStr"/>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="I268" s="7" t="inlineStr">
         <is>
-          <t>O06_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J268" s="9" t="inlineStr"/>
@@ -13605,7 +13605,7 @@
       </c>
       <c r="I269" s="7" t="inlineStr">
         <is>
-          <t>O06_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J269" s="9" t="inlineStr"/>
@@ -13654,7 +13654,7 @@
       </c>
       <c r="I270" s="7" t="inlineStr">
         <is>
-          <t>O07_Carousel3_Slide1.png, O07_Carousel3_Slide2.png, O07_Carousel3_Slide3.png, O07_Carousel3_Slide4.png, O07_Carousel3_Slide5.png, O07_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J270" s="9" t="inlineStr"/>
@@ -13703,7 +13703,7 @@
       </c>
       <c r="I271" s="7" t="inlineStr">
         <is>
-          <t>O07_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J271" s="9" t="inlineStr"/>
@@ -13752,7 +13752,7 @@
       </c>
       <c r="I272" s="7" t="inlineStr">
         <is>
-          <t>O07_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J272" s="9" t="inlineStr"/>
@@ -13801,7 +13801,7 @@
       </c>
       <c r="I273" s="7" t="inlineStr">
         <is>
-          <t>O07_Video3_Check-the-output.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J273" s="9" t="inlineStr"/>
@@ -13850,7 +13850,7 @@
       </c>
       <c r="I274" s="7" t="inlineStr">
         <is>
-          <t>O07_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J274" s="9" t="inlineStr"/>
@@ -13899,7 +13899,7 @@
       </c>
       <c r="I275" s="7" t="inlineStr">
         <is>
-          <t>O07_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J275" s="9" t="inlineStr"/>
@@ -13948,7 +13948,7 @@
       </c>
       <c r="I276" s="7" t="inlineStr">
         <is>
-          <t>O07_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J276" s="9" t="inlineStr"/>
@@ -13997,7 +13997,7 @@
       </c>
       <c r="I277" s="7" t="inlineStr">
         <is>
-          <t>O07_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J277" s="9" t="inlineStr"/>
@@ -14046,7 +14046,7 @@
       </c>
       <c r="I278" s="7" t="inlineStr">
         <is>
-          <t>O07_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J278" s="9" t="inlineStr"/>
@@ -14095,7 +14095,7 @@
       </c>
       <c r="I279" s="7" t="inlineStr">
         <is>
-          <t>O07_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J279" s="9" t="inlineStr"/>
@@ -14144,7 +14144,7 @@
       </c>
       <c r="I280" s="7" t="inlineStr">
         <is>
-          <t>O07_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J280" s="9" t="inlineStr"/>
@@ -14193,7 +14193,7 @@
       </c>
       <c r="I281" s="7" t="inlineStr">
         <is>
-          <t>O08_Carousel3_Slide1.png, O08_Carousel3_Slide2.png, O08_Carousel3_Slide3.png, O08_Carousel3_Slide4.png, O08_Carousel3_Slide5.png, O08_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J281" s="9" t="inlineStr"/>
@@ -14242,7 +14242,7 @@
       </c>
       <c r="I282" s="7" t="inlineStr">
         <is>
-          <t>O08_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J282" s="9" t="inlineStr"/>
@@ -14291,7 +14291,7 @@
       </c>
       <c r="I283" s="7" t="inlineStr">
         <is>
-          <t>O08_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J283" s="9" t="inlineStr"/>
@@ -14340,7 +14340,7 @@
       </c>
       <c r="I284" s="7" t="inlineStr">
         <is>
-          <t>O08_Video3_Follow-up.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J284" s="9" t="inlineStr"/>
@@ -14389,7 +14389,7 @@
       </c>
       <c r="I285" s="7" t="inlineStr">
         <is>
-          <t>O08_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J285" s="9" t="inlineStr"/>
@@ -14438,7 +14438,7 @@
       </c>
       <c r="I286" s="7" t="inlineStr">
         <is>
-          <t>O08_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J286" s="9" t="inlineStr"/>
@@ -14487,7 +14487,7 @@
       </c>
       <c r="I287" s="7" t="inlineStr">
         <is>
-          <t>O08_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J287" s="9" t="inlineStr"/>
@@ -14536,7 +14536,7 @@
       </c>
       <c r="I288" s="7" t="inlineStr">
         <is>
-          <t>O08_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J288" s="9" t="inlineStr"/>
@@ -14585,7 +14585,7 @@
       </c>
       <c r="I289" s="7" t="inlineStr">
         <is>
-          <t>O08_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J289" s="9" t="inlineStr"/>
@@ -14634,7 +14634,7 @@
       </c>
       <c r="I290" s="7" t="inlineStr">
         <is>
-          <t>O08_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J290" s="9" t="inlineStr"/>
@@ -14683,7 +14683,7 @@
       </c>
       <c r="I291" s="7" t="inlineStr">
         <is>
-          <t>O08_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J291" s="9" t="inlineStr"/>
@@ -14732,7 +14732,7 @@
       </c>
       <c r="I292" s="7" t="inlineStr">
         <is>
-          <t>O09_Carousel3_Slide1.png, O09_Carousel3_Slide2.png, O09_Carousel3_Slide3.png, O09_Carousel3_Slide4.png, O09_Carousel3_Slide5.png, O09_Carousel3_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J292" s="9" t="inlineStr"/>
@@ -14781,7 +14781,7 @@
       </c>
       <c r="I293" s="7" t="inlineStr">
         <is>
-          <t>O09_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J293" s="9" t="inlineStr"/>
@@ -14830,7 +14830,7 @@
       </c>
       <c r="I294" s="7" t="inlineStr">
         <is>
-          <t>O09_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J294" s="9" t="inlineStr"/>
@@ -14879,7 +14879,7 @@
       </c>
       <c r="I295" s="7" t="inlineStr">
         <is>
-          <t>O09_Video3_Write-a-brief.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J295" s="9" t="inlineStr"/>
@@ -14928,7 +14928,7 @@
       </c>
       <c r="I296" s="7" t="inlineStr">
         <is>
-          <t>O09_Post05_Value.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J296" s="9" t="inlineStr"/>
@@ -14977,7 +14977,7 @@
       </c>
       <c r="I297" s="7" t="inlineStr">
         <is>
-          <t>O09_Post03_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J297" s="9" t="inlineStr"/>
@@ -15026,7 +15026,7 @@
       </c>
       <c r="I298" s="7" t="inlineStr">
         <is>
-          <t>O09_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J298" s="9" t="inlineStr"/>
@@ -15075,7 +15075,7 @@
       </c>
       <c r="I299" s="7" t="inlineStr">
         <is>
-          <t>O09_Post10_Whats-inside.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J299" s="9" t="inlineStr"/>
@@ -15124,7 +15124,7 @@
       </c>
       <c r="I300" s="7" t="inlineStr">
         <is>
-          <t>O09_LinkedIn1.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J300" s="9" t="inlineStr"/>
@@ -15173,7 +15173,7 @@
       </c>
       <c r="I301" s="7" t="inlineStr">
         <is>
-          <t>O09_Post07_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J301" s="9" t="inlineStr"/>
@@ -15222,7 +15222,7 @@
       </c>
       <c r="I302" s="7" t="inlineStr">
         <is>
-          <t>O09_Post09_Mockup.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J302" s="9" t="inlineStr"/>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="I303" s="7" t="inlineStr">
         <is>
-          <t>O01_Carousel1_Slide1.png, O01_Carousel1_Slide2.png, O01_Carousel1_Slide3.png, O01_Carousel1_Slide4.png, O01_Carousel1_Slide5.png, O01_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J303" s="9" t="inlineStr"/>
@@ -15320,7 +15320,7 @@
       </c>
       <c r="I304" s="7" t="inlineStr">
         <is>
-          <t>O01_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J304" s="9" t="inlineStr"/>
@@ -15369,7 +15369,7 @@
       </c>
       <c r="I305" s="7" t="inlineStr">
         <is>
-          <t>O01_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J305" s="9" t="inlineStr"/>
@@ -15418,7 +15418,7 @@
       </c>
       <c r="I306" s="7" t="inlineStr">
         <is>
-          <t>O01_Video1_Price-question.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J306" s="9" t="inlineStr"/>
@@ -15467,7 +15467,7 @@
       </c>
       <c r="I307" s="7" t="inlineStr">
         <is>
-          <t>O01_Post09_Mockup.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J307" s="9" t="inlineStr"/>
@@ -15516,7 +15516,7 @@
       </c>
       <c r="I308" s="7" t="inlineStr">
         <is>
-          <t>O01_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J308" s="9" t="inlineStr"/>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="I309" s="7" t="inlineStr">
         <is>
-          <t>O01_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J309" s="9" t="inlineStr"/>
@@ -15614,7 +15614,7 @@
       </c>
       <c r="I310" s="7" t="inlineStr">
         <is>
-          <t>O01_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J310" s="9" t="inlineStr"/>
@@ -15663,7 +15663,7 @@
       </c>
       <c r="I311" s="7" t="inlineStr">
         <is>
-          <t>O01_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J311" s="9" t="inlineStr"/>
@@ -15712,7 +15712,7 @@
       </c>
       <c r="I312" s="7" t="inlineStr">
         <is>
-          <t>O01_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J312" s="9" t="inlineStr"/>
@@ -15761,7 +15761,7 @@
       </c>
       <c r="I313" s="7" t="inlineStr">
         <is>
-          <t>O01_Banner.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J313" s="9" t="inlineStr"/>
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I314" s="7" t="inlineStr">
         <is>
-          <t>O02_Carousel1_Slide1.png, O02_Carousel1_Slide2.png, O02_Carousel1_Slide3.png, O02_Carousel1_Slide4.png, O02_Carousel1_Slide5.png, O02_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J314" s="9" t="inlineStr"/>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="I315" s="7" t="inlineStr">
         <is>
-          <t>O02_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J315" s="9" t="inlineStr"/>
@@ -15908,7 +15908,7 @@
       </c>
       <c r="I316" s="7" t="inlineStr">
         <is>
-          <t>O02_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J316" s="9" t="inlineStr"/>
@@ -15957,7 +15957,7 @@
       </c>
       <c r="I317" s="7" t="inlineStr">
         <is>
-          <t>O02_Video1_Ten-second-test.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J317" s="9" t="inlineStr"/>
@@ -16006,7 +16006,7 @@
       </c>
       <c r="I318" s="7" t="inlineStr">
         <is>
-          <t>O02_Banner.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J318" s="9" t="inlineStr"/>
@@ -16055,7 +16055,7 @@
       </c>
       <c r="I319" s="7" t="inlineStr">
         <is>
-          <t>O02_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J319" s="9" t="inlineStr"/>
@@ -16104,7 +16104,7 @@
       </c>
       <c r="I320" s="7" t="inlineStr">
         <is>
-          <t>O02_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J320" s="9" t="inlineStr"/>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="I321" s="7" t="inlineStr">
         <is>
-          <t>O02_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J321" s="9" t="inlineStr"/>
@@ -16202,7 +16202,7 @@
       </c>
       <c r="I322" s="7" t="inlineStr">
         <is>
-          <t>O02_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J322" s="9" t="inlineStr"/>
@@ -16251,7 +16251,7 @@
       </c>
       <c r="I323" s="7" t="inlineStr">
         <is>
-          <t>O02_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J323" s="9" t="inlineStr"/>
@@ -16300,7 +16300,7 @@
       </c>
       <c r="I324" s="7" t="inlineStr">
         <is>
-          <t>O02_Post05_Value.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J324" s="9" t="inlineStr"/>
@@ -16349,7 +16349,7 @@
       </c>
       <c r="I325" s="7" t="inlineStr">
         <is>
-          <t>O03_Carousel1_Slide1.png, O03_Carousel1_Slide2.png, O03_Carousel1_Slide3.png, O03_Carousel1_Slide4.png, O03_Carousel1_Slide5.png, O03_Carousel1_Slide6.png</t>
+          <t>Post_01_0800_Instagram-and-Facebook-feed_Carousel-or-tip-post</t>
         </is>
       </c>
       <c r="J325" s="9" t="inlineStr"/>
@@ -16398,7 +16398,7 @@
       </c>
       <c r="I326" s="7" t="inlineStr">
         <is>
-          <t>O03_Post02_Launch.png</t>
+          <t>Post_02_0900_WhatsApp-Status_Launch-promo-post</t>
         </is>
       </c>
       <c r="J326" s="9" t="inlineStr"/>
@@ -16447,7 +16447,7 @@
       </c>
       <c r="I327" s="7" t="inlineStr">
         <is>
-          <t>O03_Story1_New.png</t>
+          <t>Post_03_1030_Instagram-Story_New-offer-story</t>
         </is>
       </c>
       <c r="J327" s="9" t="inlineStr"/>
@@ -16496,7 +16496,7 @@
       </c>
       <c r="I328" s="7" t="inlineStr">
         <is>
-          <t>O03_Video1_Four-pillars.mp4</t>
+          <t>Post_04_1230_Instagram-Reel-and-Facebook-video_Short-video</t>
         </is>
       </c>
       <c r="J328" s="9" t="inlineStr"/>
@@ -16545,7 +16545,7 @@
       </c>
       <c r="I329" s="7" t="inlineStr">
         <is>
-          <t>O03_Banner.png</t>
+          <t>Post_05_1330_WhatsApp-Status_What-is-inside</t>
         </is>
       </c>
       <c r="J329" s="9" t="inlineStr"/>
@@ -16594,7 +16594,7 @@
       </c>
       <c r="I330" s="7" t="inlineStr">
         <is>
-          <t>O03_Post08_Honest-answer.png</t>
+          <t>Post_06_1500_Facebook-feed_Honest-answer-objection-post</t>
         </is>
       </c>
       <c r="J330" s="9" t="inlineStr"/>
@@ -16643,7 +16643,7 @@
       </c>
       <c r="I331" s="7" t="inlineStr">
         <is>
-          <t>O03_Story2_Price.png</t>
+          <t>Post_07_1600_Instagram-Story_Price-story</t>
         </is>
       </c>
       <c r="J331" s="9" t="inlineStr"/>
@@ -16692,7 +16692,7 @@
       </c>
       <c r="I332" s="7" t="inlineStr">
         <is>
-          <t>O03_Post06_Order.png</t>
+          <t>Post_08_1700_WhatsApp-Status_Direct-response-post</t>
         </is>
       </c>
       <c r="J332" s="9" t="inlineStr"/>
@@ -16741,7 +16741,7 @@
       </c>
       <c r="I333" s="7" t="inlineStr">
         <is>
-          <t>O03_LinkedIn2.txt</t>
+          <t>Post_09_1830_LinkedIn_Text-post-no-media-needed</t>
         </is>
       </c>
       <c r="J333" s="9" t="inlineStr"/>
@@ -16790,7 +16790,7 @@
       </c>
       <c r="I334" s="7" t="inlineStr">
         <is>
-          <t>O03_Post01_Tip.png</t>
+          <t>Post_10_2000_Instagram-and-Facebook-feed_Second-feed-post</t>
         </is>
       </c>
       <c r="J334" s="9" t="inlineStr"/>
@@ -16839,7 +16839,7 @@
       </c>
       <c r="I335" s="7" t="inlineStr">
         <is>
-          <t>O03_Post05_Value.png</t>
+          <t>Post_11_2100_WhatsApp-Status_Banner-or-price-graphic</t>
         </is>
       </c>
       <c r="J335" s="9" t="inlineStr"/>

</xml_diff>